<commit_message>
added retry and reports to integration
</commit_message>
<xml_diff>
--- a/src/test/resources/Testdata.xlsx
+++ b/src/test/resources/Testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d0bfd4e7872013d0/Desktop/SDET Class/Testng/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="8_{78179A37-ECA0-47E1-AB70-F80F6F4BF4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{221F3166-65D5-49B3-82EF-80913516143E}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{DB4D6F9C-ED1C-421A-9C61-775E16A580AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BB5FE28-0E5B-47FE-8496-CF5BB7676E26}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9EB3E75D-3105-4D9D-A75D-FDEFFD928651}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{9EB3E75D-3105-4D9D-A75D-FDEFFD928651}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="24">
   <si>
     <t>Username</t>
   </si>
@@ -81,6 +81,33 @@
   </si>
   <si>
     <t>valid</t>
+  </si>
+  <si>
+    <t>onlyusername</t>
+  </si>
+  <si>
+    <t>onlypassword</t>
+  </si>
+  <si>
+    <t>onlypasswordconfirm</t>
+  </si>
+  <si>
+    <t>onlypassandconfirm</t>
+  </si>
+  <si>
+    <t>wrongpasswordconfirm</t>
+  </si>
+  <si>
+    <t>invalidpassword</t>
+  </si>
+  <si>
+    <t>usernamespace</t>
+  </si>
+  <si>
+    <t>validregister</t>
+  </si>
+  <si>
+    <t>dsalgoprojectcomp</t>
   </si>
 </sst>
 </file>
@@ -582,12 +609,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9BB40C1-0636-4AB5-A896-5008C2AF0E1E}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -608,28 +636,91 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>24680</v>
+      </c>
+      <c r="C7">
+        <v>24680</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -642,7 +733,7 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="59.21875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="59.33203125" style="6" customWidth="1"/>
     <col min="2" max="2" width="34.5546875" style="6" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>